<commit_message>
updates for region and project awareness
</commit_message>
<xml_diff>
--- a/Requisitioner.xlsx
+++ b/Requisitioner.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\N-20W1PF3VP3VC-Data\rabanes\Downloads\Raawa Generator_3\Raawa Generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8151C95-6C66-404F-8668-17B9177C24A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A703E82-B7B3-4F17-A51F-22150D8616E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
   <si>
     <t>Requisitioner</t>
   </si>
@@ -79,6 +90,18 @@
   </si>
   <si>
     <t>MIN</t>
+  </si>
+  <si>
+    <t>EUL MIGRATION - ADVANCE SURVEY</t>
+  </si>
+  <si>
+    <t>Miguel Evangelista</t>
+  </si>
+  <si>
+    <t>NTG/B&amp;D/NBSD</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 09176884753</t>
   </si>
 </sst>
 </file>
@@ -462,7 +485,7 @@
     <col min="2" max="2" width="27.26953125" customWidth="1"/>
     <col min="3" max="4" width="28" customWidth="1"/>
     <col min="5" max="5" width="18.26953125" customWidth="1"/>
-    <col min="6" max="6" width="26.36328125" customWidth="1"/>
+    <col min="6" max="6" width="32.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -542,22 +565,50 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
+      <c r="A5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="1">
+        <v>10009038</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
+      <c r="A6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="1">
+        <v>10009038</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>

</xml_diff>